<commit_message>
feat: incorporar 6 reglas de negocio confirmadas (hojas de control, código certificado, docente COIN y ciclo)
</commit_message>
<xml_diff>
--- a/tests/fixtures/synthetic_control_aulas.xlsx
+++ b/tests/fixtures/synthetic_control_aulas.xlsx
@@ -7,7 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control_Aulas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla_CMI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla_ABBUEI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla_GICE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla_EPA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla_LATEX" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla_IPI" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla_UEI" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla_CAI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creación aulas GDA" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONTROL" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,6 +429,178 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -743,4 +924,606 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO DE AULA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CURSO QUE REALIZA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PROGRAMA ACADÉMICO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CATÁLOGO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CLASE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NOMBRE DE LA SECCIÓN</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>DOCENTE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>FECHA DE INICIO DEL CURSO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FECHA DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FECHA 2 DE FINALIZACIÓN DEL CURSO</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ENVÍO DE NOTAS A PROFESORES</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS Y CIERRE DE CURSO</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>CERTIFICADOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>